<commit_message>
data(aud): daily refresh 2026-09-17T07:57Z
</commit_message>
<xml_diff>
--- a/history/aud/aofm_tib_issuance.xlsx
+++ b/history/aud/aofm_tib_issuance.xlsx
@@ -24703,7 +24703,7 @@
         <v>46258</v>
       </c>
     </row>
-    <row r="426" ht="16.95" customHeight="0">
+    <row r="426" ht="17" customHeight="0">
       <c s="3" r="A426">
         <v>46268</v>
       </c>
@@ -24769,7 +24769,72 @@
         <v>46272</v>
       </c>
     </row>
-    <row r="427" ht="0.05" customHeight="1"/>
+    <row r="427" ht="17" customHeight="0">
+      <c s="3" r="A427">
+        <v>46282</v>
+      </c>
+      <c s="4" t="inlineStr" r="B427">
+        <is>
+          <t xml:space="preserve">TIB309</t>
+        </is>
+      </c>
+      <c s="3" r="C427">
+        <v>51369</v>
+      </c>
+      <c s="5" r="D427">
+        <v>1.25</v>
+      </c>
+      <c s="4" t="inlineStr" r="E427">
+        <is>
+          <t xml:space="preserve">AU000XCLWAO6    </t>
+        </is>
+      </c>
+      <c s="7" r="F427">
+        <v>100000000.0000</v>
+      </c>
+      <c s="7" r="G427">
+        <v>100000000.0000</v>
+      </c>
+      <c s="7" r="H427">
+        <v>447000000.0000</v>
+      </c>
+      <c s="11" r="I427">
+        <v>4.47</v>
+      </c>
+      <c s="8" r="J427">
+        <v>3.164125</v>
+      </c>
+      <c s="9" r="K427">
+        <v>3.1625</v>
+      </c>
+      <c s="9" r="L427">
+        <v>3.1675</v>
+      </c>
+      <c s="9" r="M427">
+        <v>3.225</v>
+      </c>
+      <c s="9" r="N427">
+        <v>3.17578859060403</v>
+      </c>
+      <c s="8" r="O427">
+        <v>3.1738</v>
+      </c>
+      <c s="7" r="P427">
+        <v>45</v>
+      </c>
+      <c s="7" r="Q427">
+        <v>10</v>
+      </c>
+      <c s="7" r="R427">
+        <v>6</v>
+      </c>
+      <c s="7" r="S427">
+        <v>107899900.0000</v>
+      </c>
+      <c s="10" r="T427">
+        <v>46286</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells>
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
data(aud): daily refresh 2026-10-08T09:23Z
</commit_message>
<xml_diff>
--- a/history/aud/aofm_tib_issuance.xlsx
+++ b/history/aud/aofm_tib_issuance.xlsx
@@ -785,27 +785,19 @@
         </is>
       </c>
       <c s="3" r="C12">
-        <v>34931</v>
+        <v>38584</v>
       </c>
       <c s="5" r="D12">
-        <v>4</v>
+        <v>4.75</v>
       </c>
       <c s="4" t="str" r="E12"/>
       <c s="6" t="str" r="F12"/>
-      <c s="7" r="G12">
-        <v>15700000.0000</v>
-      </c>
+      <c s="6" t="str" r="G12"/>
       <c s="6" t="str" r="H12"/>
       <c s="6" t="str" r="I12"/>
-      <c s="8" r="J12">
-        <v>6.606</v>
-      </c>
-      <c s="9" r="K12">
-        <v>5.29</v>
-      </c>
-      <c s="9" r="L12">
-        <v>7</v>
-      </c>
+      <c s="6" t="str" r="J12"/>
+      <c s="6" t="str" r="K12"/>
+      <c s="6" t="str" r="L12"/>
       <c s="6" t="str" r="M12"/>
       <c s="6" t="str" r="N12"/>
       <c s="6" t="str" r="O12"/>
@@ -827,30 +819,26 @@
         </is>
       </c>
       <c s="3" r="C13">
-        <v>38584</v>
+        <v>34931</v>
       </c>
       <c s="5" r="D13">
         <v>4</v>
       </c>
-      <c s="4" t="inlineStr" r="E13">
-        <is>
-          <t xml:space="preserve">AU0000XCLSO9</t>
-        </is>
-      </c>
+      <c s="4" t="str" r="E13"/>
       <c s="6" t="str" r="F13"/>
       <c s="7" r="G13">
-        <v>50100000.0000</v>
+        <v>15700000.0000</v>
       </c>
       <c s="6" t="str" r="H13"/>
       <c s="6" t="str" r="I13"/>
       <c s="8" r="J13">
-        <v>4.972</v>
+        <v>6.606</v>
       </c>
       <c s="9" r="K13">
-        <v>4.88</v>
+        <v>5.29</v>
       </c>
       <c s="9" r="L13">
-        <v>4.98</v>
+        <v>7</v>
       </c>
       <c s="6" t="str" r="M13"/>
       <c s="6" t="str" r="N13"/>
@@ -858,9 +846,7 @@
       <c s="6" t="str" r="P13"/>
       <c s="6" t="str" r="Q13"/>
       <c s="6" t="str" r="R13"/>
-      <c s="7" r="S13">
-        <v>44713937.0000</v>
-      </c>
+      <c s="6" t="str" r="S13"/>
       <c s="10" r="T13">
         <v>31358</v>
       </c>
@@ -875,26 +861,40 @@
         </is>
       </c>
       <c s="3" r="C14">
-        <v>34931</v>
+        <v>38584</v>
       </c>
       <c s="5" r="D14">
-        <v>6.25</v>
-      </c>
-      <c s="4" t="str" r="E14"/>
+        <v>4</v>
+      </c>
+      <c s="4" t="inlineStr" r="E14">
+        <is>
+          <t xml:space="preserve">AU0000XCLSO9</t>
+        </is>
+      </c>
       <c s="6" t="str" r="F14"/>
-      <c s="6" t="str" r="G14"/>
+      <c s="7" r="G14">
+        <v>50100000.0000</v>
+      </c>
       <c s="6" t="str" r="H14"/>
       <c s="6" t="str" r="I14"/>
-      <c s="6" t="str" r="J14"/>
-      <c s="6" t="str" r="K14"/>
-      <c s="6" t="str" r="L14"/>
+      <c s="8" r="J14">
+        <v>4.972</v>
+      </c>
+      <c s="9" r="K14">
+        <v>4.88</v>
+      </c>
+      <c s="9" r="L14">
+        <v>4.98</v>
+      </c>
       <c s="6" t="str" r="M14"/>
       <c s="6" t="str" r="N14"/>
       <c s="6" t="str" r="O14"/>
       <c s="6" t="str" r="P14"/>
       <c s="6" t="str" r="Q14"/>
       <c s="6" t="str" r="R14"/>
-      <c s="6" t="str" r="S14"/>
+      <c s="7" r="S14">
+        <v>44713937.0000</v>
+      </c>
       <c s="10" r="T14">
         <v>31358</v>
       </c>
@@ -909,10 +909,10 @@
         </is>
       </c>
       <c s="3" r="C15">
-        <v>38584</v>
+        <v>34931</v>
       </c>
       <c s="5" r="D15">
-        <v>4.75</v>
+        <v>6.25</v>
       </c>
       <c s="4" t="str" r="E15"/>
       <c s="6" t="str" r="F15"/>
@@ -2192,11 +2192,13 @@
         <v>34931</v>
       </c>
       <c s="5" r="D48">
-        <v>4</v>
+        <v>5.7</v>
       </c>
       <c s="4" t="str" r="E48"/>
       <c s="6" t="str" r="F48"/>
-      <c s="6" t="str" r="G48"/>
+      <c s="7" r="G48">
+        <v>200000.0000</v>
+      </c>
       <c s="6" t="str" r="H48"/>
       <c s="6" t="str" r="I48"/>
       <c s="8" r="J48">
@@ -2228,15 +2230,13 @@
         <v>38584</v>
       </c>
       <c s="5" r="D49">
-        <v>4</v>
-      </c>
-      <c s="4" t="inlineStr" r="E49">
-        <is>
-          <t xml:space="preserve">AU0000XCLSO9</t>
-        </is>
-      </c>
+        <v>5.5</v>
+      </c>
+      <c s="4" t="str" r="E49"/>
       <c s="6" t="str" r="F49"/>
-      <c s="6" t="str" r="G49"/>
+      <c s="7" r="G49">
+        <v>300000.0000</v>
+      </c>
       <c s="6" t="str" r="H49"/>
       <c s="6" t="str" r="I49"/>
       <c s="8" r="J49">
@@ -2268,13 +2268,11 @@
         <v>34931</v>
       </c>
       <c s="5" r="D50">
-        <v>5.7</v>
+        <v>4</v>
       </c>
       <c s="4" t="str" r="E50"/>
       <c s="6" t="str" r="F50"/>
-      <c s="7" r="G50">
-        <v>200000.0000</v>
-      </c>
+      <c s="6" t="str" r="G50"/>
       <c s="6" t="str" r="H50"/>
       <c s="6" t="str" r="I50"/>
       <c s="8" r="J50">
@@ -2306,13 +2304,15 @@
         <v>38584</v>
       </c>
       <c s="5" r="D51">
-        <v>5.5</v>
-      </c>
-      <c s="4" t="str" r="E51"/>
+        <v>4</v>
+      </c>
+      <c s="4" t="inlineStr" r="E51">
+        <is>
+          <t xml:space="preserve">AU0000XCLSO9</t>
+        </is>
+      </c>
       <c s="6" t="str" r="F51"/>
-      <c s="7" r="G51">
-        <v>300000.0000</v>
-      </c>
+      <c s="6" t="str" r="G51"/>
       <c s="6" t="str" r="H51"/>
       <c s="6" t="str" r="I51"/>
       <c s="8" r="J51">
@@ -20181,57 +20181,57 @@
         </is>
       </c>
       <c s="3" r="C358">
-        <v>46712</v>
+        <v>51369</v>
       </c>
       <c s="5" r="D358">
-        <v>0.75</v>
+        <v>1.25</v>
       </c>
       <c s="4" t="inlineStr" r="E358">
         <is>
-          <t xml:space="preserve">AU000XCLWAV1</t>
+          <t xml:space="preserve">AU000XCLWAO6</t>
         </is>
       </c>
       <c s="7" r="F358">
-        <v>100000000.0000</v>
+        <v>50000000.0000</v>
       </c>
       <c s="7" r="G358">
-        <v>100000000.0000</v>
+        <v>50000000.0000</v>
       </c>
       <c s="7" r="H358">
-        <v>390000000.0000</v>
+        <v>169000000.0000</v>
       </c>
       <c s="11" r="I358">
-        <v>3.9</v>
+        <v>3.38</v>
       </c>
       <c s="8" r="J358">
-        <v>1.098125</v>
+        <v>1.6388</v>
       </c>
       <c s="9" r="K358">
-        <v>1.085</v>
+        <v>1.62</v>
       </c>
       <c s="9" r="L358">
-        <v>1.11</v>
+        <v>1.65</v>
       </c>
       <c s="9" r="M358">
-        <v>1.25</v>
+        <v>1.85</v>
       </c>
       <c s="9" r="N358">
-        <v>1.1216858974359</v>
+        <v>1.68596153846154</v>
       </c>
       <c s="8" r="O358">
-        <v>1.1162</v>
+        <v>1.6415</v>
       </c>
       <c s="7" r="P358">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c s="7" r="Q358">
+        <v>16</v>
+      </c>
+      <c s="7" r="R358">
         <v>13</v>
       </c>
-      <c s="7" r="R358">
-        <v>10</v>
-      </c>
       <c s="7" r="S358">
-        <v>116811500.0000</v>
+        <v>57837210.0000</v>
       </c>
       <c s="10" r="T358">
         <v>45106</v>
@@ -20247,57 +20247,57 @@
         </is>
       </c>
       <c s="3" r="C359">
-        <v>51369</v>
+        <v>46712</v>
       </c>
       <c s="5" r="D359">
+        <v>0.75</v>
+      </c>
+      <c s="4" t="inlineStr" r="E359">
+        <is>
+          <t xml:space="preserve">AU000XCLWAV1</t>
+        </is>
+      </c>
+      <c s="7" r="F359">
+        <v>100000000.0000</v>
+      </c>
+      <c s="7" r="G359">
+        <v>100000000.0000</v>
+      </c>
+      <c s="7" r="H359">
+        <v>390000000.0000</v>
+      </c>
+      <c s="11" r="I359">
+        <v>3.9</v>
+      </c>
+      <c s="8" r="J359">
+        <v>1.098125</v>
+      </c>
+      <c s="9" r="K359">
+        <v>1.085</v>
+      </c>
+      <c s="9" r="L359">
+        <v>1.11</v>
+      </c>
+      <c s="9" r="M359">
         <v>1.25</v>
       </c>
-      <c s="4" t="inlineStr" r="E359">
-        <is>
-          <t xml:space="preserve">AU000XCLWAO6</t>
-        </is>
-      </c>
-      <c s="7" r="F359">
-        <v>50000000.0000</v>
-      </c>
-      <c s="7" r="G359">
-        <v>50000000.0000</v>
-      </c>
-      <c s="7" r="H359">
-        <v>169000000.0000</v>
-      </c>
-      <c s="11" r="I359">
-        <v>3.38</v>
-      </c>
-      <c s="8" r="J359">
-        <v>1.6388</v>
-      </c>
-      <c s="9" r="K359">
-        <v>1.62</v>
-      </c>
-      <c s="9" r="L359">
-        <v>1.65</v>
-      </c>
-      <c s="9" r="M359">
-        <v>1.85</v>
-      </c>
       <c s="9" r="N359">
-        <v>1.68596153846154</v>
+        <v>1.1216858974359</v>
       </c>
       <c s="8" r="O359">
-        <v>1.6415</v>
+        <v>1.1162</v>
       </c>
       <c s="7" r="P359">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c s="7" r="Q359">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c s="7" r="R359">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c s="7" r="S359">
-        <v>57837210.0000</v>
+        <v>116811500.0000</v>
       </c>
       <c s="10" r="T359">
         <v>45106</v>
@@ -20379,48 +20379,48 @@
         </is>
       </c>
       <c s="3" r="C361">
-        <v>47746</v>
+        <v>51369</v>
       </c>
       <c s="5" r="D361">
-        <v>2.5</v>
+        <v>1.25</v>
       </c>
       <c s="4" t="inlineStr" r="E361">
         <is>
-          <t xml:space="preserve">AU0000XCLWV6</t>
+          <t xml:space="preserve">AU000XCLWAO6</t>
         </is>
       </c>
       <c s="7" r="F361">
-        <v>100000000.0000</v>
+        <v>50000000.0000</v>
       </c>
       <c s="7" r="G361">
-        <v>100000000.0000</v>
+        <v>50000000.0000</v>
       </c>
       <c s="7" r="H361">
-        <v>355000000.0000</v>
+        <v>175000000.0000</v>
       </c>
       <c s="11" r="I361">
-        <v>3.55</v>
+        <v>3.5</v>
       </c>
       <c s="8" r="J361">
-        <v>1.41525</v>
+        <v>1.8125</v>
       </c>
       <c s="9" r="K361">
-        <v>1.405</v>
+        <v>1.8</v>
       </c>
       <c s="9" r="L361">
-        <v>1.42</v>
+        <v>1.82</v>
       </c>
       <c s="9" r="M361">
-        <v>1.5</v>
+        <v>1.9225</v>
       </c>
       <c s="9" r="N361">
-        <v>1.43426056338028</v>
+        <v>1.84494285714286</v>
       </c>
       <c s="8" r="O361">
-        <v>1.4289</v>
+        <v>1.8265</v>
       </c>
       <c s="7" r="P361">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c s="7" r="Q361">
         <v>13</v>
@@ -20429,7 +20429,7 @@
         <v>8</v>
       </c>
       <c s="7" r="S361">
-        <v>148765500.0000</v>
+        <v>56858550.0000</v>
       </c>
       <c s="10" r="T361">
         <v>45148</v>
@@ -20445,48 +20445,48 @@
         </is>
       </c>
       <c s="3" r="C362">
-        <v>51369</v>
+        <v>47746</v>
       </c>
       <c s="5" r="D362">
-        <v>1.25</v>
+        <v>2.5</v>
       </c>
       <c s="4" t="inlineStr" r="E362">
         <is>
-          <t xml:space="preserve">AU000XCLWAO6</t>
+          <t xml:space="preserve">AU0000XCLWV6</t>
         </is>
       </c>
       <c s="7" r="F362">
-        <v>50000000.0000</v>
+        <v>100000000.0000</v>
       </c>
       <c s="7" r="G362">
-        <v>50000000.0000</v>
+        <v>100000000.0000</v>
       </c>
       <c s="7" r="H362">
-        <v>175000000.0000</v>
+        <v>355000000.0000</v>
       </c>
       <c s="11" r="I362">
-        <v>3.5</v>
+        <v>3.55</v>
       </c>
       <c s="8" r="J362">
-        <v>1.8125</v>
+        <v>1.41525</v>
       </c>
       <c s="9" r="K362">
-        <v>1.8</v>
+        <v>1.405</v>
       </c>
       <c s="9" r="L362">
-        <v>1.82</v>
+        <v>1.42</v>
       </c>
       <c s="9" r="M362">
-        <v>1.9225</v>
+        <v>1.5</v>
       </c>
       <c s="9" r="N362">
-        <v>1.84494285714286</v>
+        <v>1.43426056338028</v>
       </c>
       <c s="8" r="O362">
-        <v>1.8265</v>
+        <v>1.4289</v>
       </c>
       <c s="7" r="P362">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c s="7" r="Q362">
         <v>13</v>
@@ -20495,7 +20495,7 @@
         <v>8</v>
       </c>
       <c s="7" r="S362">
-        <v>56858550.0000</v>
+        <v>148765500.0000</v>
       </c>
       <c s="10" r="T362">
         <v>45148</v>
@@ -20841,57 +20841,57 @@
         </is>
       </c>
       <c s="3" r="C368">
-        <v>47746</v>
+        <v>54840</v>
       </c>
       <c s="5" r="D368">
-        <v>2.5</v>
+        <v>1</v>
       </c>
       <c s="4" t="inlineStr" r="E368">
         <is>
-          <t xml:space="preserve">AU0000XCLWV6</t>
+          <t xml:space="preserve">AU0000024044</t>
         </is>
       </c>
       <c s="7" r="F368">
-        <v>100000000.0000</v>
+        <v>50000000.0000</v>
       </c>
       <c s="7" r="G368">
-        <v>100000000.0000</v>
+        <v>50000000.0000</v>
       </c>
       <c s="7" r="H368">
-        <v>220000000.0000</v>
+        <v>228000000.0000</v>
       </c>
       <c s="11" r="I368">
-        <v>2.2</v>
+        <v>4.56</v>
       </c>
       <c s="8" r="J368">
-        <v>1.774425</v>
+        <v>2.21575</v>
       </c>
       <c s="9" r="K368">
-        <v>1.7625</v>
+        <v>2.2025</v>
       </c>
       <c s="9" r="L368">
-        <v>1.79</v>
+        <v>2.23</v>
       </c>
       <c s="9" r="M368">
-        <v>1.87</v>
+        <v>2.33</v>
       </c>
       <c s="9" r="N368">
-        <v>1.80184090909091</v>
+        <v>2.24574561403509</v>
       </c>
       <c s="8" r="O368">
-        <v>1.776</v>
+        <v>2.2542</v>
       </c>
       <c s="7" r="P368">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c s="7" r="Q368">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c s="7" r="R368">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c s="7" r="S368">
-        <v>147568290.0000</v>
+        <v>45060490.0000</v>
       </c>
       <c s="10" r="T368">
         <v>45260</v>
@@ -20907,57 +20907,57 @@
         </is>
       </c>
       <c s="3" r="C369">
-        <v>54840</v>
+        <v>47746</v>
       </c>
       <c s="5" r="D369">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c s="4" t="inlineStr" r="E369">
         <is>
-          <t xml:space="preserve">AU0000024044</t>
+          <t xml:space="preserve">AU0000XCLWV6</t>
         </is>
       </c>
       <c s="7" r="F369">
-        <v>50000000.0000</v>
+        <v>100000000.0000</v>
       </c>
       <c s="7" r="G369">
-        <v>50000000.0000</v>
+        <v>100000000.0000</v>
       </c>
       <c s="7" r="H369">
-        <v>228000000.0000</v>
+        <v>220000000.0000</v>
       </c>
       <c s="11" r="I369">
-        <v>4.56</v>
+        <v>2.2</v>
       </c>
       <c s="8" r="J369">
-        <v>2.21575</v>
+        <v>1.774425</v>
       </c>
       <c s="9" r="K369">
-        <v>2.2025</v>
+        <v>1.7625</v>
       </c>
       <c s="9" r="L369">
-        <v>2.23</v>
+        <v>1.79</v>
       </c>
       <c s="9" r="M369">
-        <v>2.33</v>
+        <v>1.87</v>
       </c>
       <c s="9" r="N369">
-        <v>2.24574561403509</v>
+        <v>1.80184090909091</v>
       </c>
       <c s="8" r="O369">
-        <v>2.2542</v>
+        <v>1.776</v>
       </c>
       <c s="7" r="P369">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c s="7" r="Q369">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c s="7" r="R369">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c s="7" r="S369">
-        <v>45060490.0000</v>
+        <v>147568290.0000</v>
       </c>
       <c s="10" r="T369">
         <v>45260</v>
@@ -21457,57 +21457,57 @@
         </is>
       </c>
       <c s="3" r="C377">
-        <v>49542</v>
+        <v>54840</v>
       </c>
       <c s="5" r="D377">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c s="4" t="inlineStr" r="E377">
         <is>
-          <t xml:space="preserve">AU000XCLWAF4</t>
+          <t xml:space="preserve">AU0000024044</t>
         </is>
       </c>
       <c s="7" r="F377">
-        <v>100000000.0000</v>
+        <v>50000000.0000</v>
       </c>
       <c s="7" r="G377">
-        <v>100000000.0000</v>
+        <v>50000000.0000</v>
       </c>
       <c s="7" r="H377">
-        <v>390000000.0000</v>
+        <v>191000000.0000</v>
       </c>
       <c s="11" r="I377">
-        <v>3.9</v>
+        <v>3.82</v>
       </c>
       <c s="8" r="J377">
-        <v>1.973875</v>
+        <v>2.1971</v>
       </c>
       <c s="9" r="K377">
-        <v>1.9675</v>
+        <v>2.1825</v>
       </c>
       <c s="9" r="L377">
-        <v>1.9775</v>
+        <v>2.21</v>
       </c>
       <c s="9" r="M377">
-        <v>2.045</v>
+        <v>2.315</v>
       </c>
       <c s="9" r="N377">
-        <v>1.99477564102564</v>
+        <v>2.23082460732984</v>
       </c>
       <c s="8" r="O377">
-        <v>1.993</v>
+        <v>2.2155</v>
       </c>
       <c s="7" r="P377">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c s="7" r="Q377">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c s="7" r="R377">
         <v>8</v>
       </c>
       <c s="7" r="S377">
-        <v>133726300.0000</v>
+        <v>46408130.0000</v>
       </c>
       <c s="10" r="T377">
         <v>45456</v>
@@ -21523,57 +21523,57 @@
         </is>
       </c>
       <c s="3" r="C378">
-        <v>54840</v>
+        <v>49542</v>
       </c>
       <c s="5" r="D378">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c s="4" t="inlineStr" r="E378">
         <is>
-          <t xml:space="preserve">AU0000024044</t>
+          <t xml:space="preserve">AU000XCLWAF4</t>
         </is>
       </c>
       <c s="7" r="F378">
-        <v>50000000.0000</v>
+        <v>100000000.0000</v>
       </c>
       <c s="7" r="G378">
-        <v>50000000.0000</v>
+        <v>100000000.0000</v>
       </c>
       <c s="7" r="H378">
-        <v>191000000.0000</v>
+        <v>390000000.0000</v>
       </c>
       <c s="11" r="I378">
-        <v>3.82</v>
+        <v>3.9</v>
       </c>
       <c s="8" r="J378">
-        <v>2.1971</v>
+        <v>1.973875</v>
       </c>
       <c s="9" r="K378">
-        <v>2.1825</v>
+        <v>1.9675</v>
       </c>
       <c s="9" r="L378">
-        <v>2.21</v>
+        <v>1.9775</v>
       </c>
       <c s="9" r="M378">
-        <v>2.315</v>
+        <v>2.045</v>
       </c>
       <c s="9" r="N378">
-        <v>2.23082460732984</v>
+        <v>1.99477564102564</v>
       </c>
       <c s="8" r="O378">
-        <v>2.2155</v>
+        <v>1.993</v>
       </c>
       <c s="7" r="P378">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c s="7" r="Q378">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c s="7" r="R378">
         <v>8</v>
       </c>
       <c s="7" r="S378">
-        <v>46408130.0000</v>
+        <v>133726300.0000</v>
       </c>
       <c s="10" r="T378">
         <v>45456</v>
@@ -21985,57 +21985,57 @@
         </is>
       </c>
       <c s="3" r="C385">
-        <v>49542</v>
+        <v>54840</v>
       </c>
       <c s="5" r="D385">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c s="4" t="inlineStr" r="E385">
         <is>
-          <t xml:space="preserve">AU000XCLWAF4</t>
+          <t xml:space="preserve">AU0000024044</t>
         </is>
       </c>
       <c s="7" r="F385">
-        <v>100000000.0000</v>
+        <v>50000000.0000</v>
       </c>
       <c s="7" r="G385">
-        <v>100000000.0000</v>
+        <v>50000000.0000</v>
       </c>
       <c s="7" r="H385">
-        <v>290000000.0000</v>
+        <v>143000000.0000</v>
       </c>
       <c s="11" r="I385">
-        <v>2.9</v>
+        <v>2.86</v>
       </c>
       <c s="8" r="J385">
-        <v>1.67625</v>
+        <v>2.0167</v>
       </c>
       <c s="9" r="K385">
-        <v>1.665</v>
+        <v>2.01</v>
       </c>
       <c s="9" r="L385">
-        <v>1.6825</v>
+        <v>2.0225</v>
       </c>
       <c s="9" r="M385">
-        <v>1.7275</v>
+        <v>2.0775</v>
       </c>
       <c s="9" r="N385">
-        <v>1.69258620689655</v>
+        <v>2.03480769230769</v>
       </c>
       <c s="8" r="O385">
-        <v>1.6785</v>
+        <v>2.0325</v>
       </c>
       <c s="7" r="P385">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c s="7" r="Q385">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c s="7" r="R385">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c s="7" r="S385">
-        <v>139253000.0000</v>
+        <v>48944460.0000</v>
       </c>
       <c s="10" r="T385">
         <v>45568</v>
@@ -22051,57 +22051,57 @@
         </is>
       </c>
       <c s="3" r="C386">
-        <v>54840</v>
+        <v>49542</v>
       </c>
       <c s="5" r="D386">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c s="4" t="inlineStr" r="E386">
         <is>
-          <t xml:space="preserve">AU0000024044</t>
+          <t xml:space="preserve">AU000XCLWAF4</t>
         </is>
       </c>
       <c s="7" r="F386">
-        <v>50000000.0000</v>
+        <v>100000000.0000</v>
       </c>
       <c s="7" r="G386">
-        <v>50000000.0000</v>
+        <v>100000000.0000</v>
       </c>
       <c s="7" r="H386">
-        <v>143000000.0000</v>
+        <v>290000000.0000</v>
       </c>
       <c s="11" r="I386">
-        <v>2.86</v>
+        <v>2.9</v>
       </c>
       <c s="8" r="J386">
-        <v>2.0167</v>
+        <v>1.67625</v>
       </c>
       <c s="9" r="K386">
-        <v>2.01</v>
+        <v>1.665</v>
       </c>
       <c s="9" r="L386">
-        <v>2.0225</v>
+        <v>1.6825</v>
       </c>
       <c s="9" r="M386">
-        <v>2.0775</v>
+        <v>1.7275</v>
       </c>
       <c s="9" r="N386">
-        <v>2.03480769230769</v>
+        <v>1.69258620689655</v>
       </c>
       <c s="8" r="O386">
-        <v>2.0325</v>
+        <v>1.6785</v>
       </c>
       <c s="7" r="P386">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c s="7" r="Q386">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c s="7" r="R386">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c s="7" r="S386">
-        <v>48944460.0000</v>
+        <v>139253000.0000</v>
       </c>
       <c s="10" r="T386">
         <v>45568</v>
@@ -24833,6 +24833,72 @@
       </c>
       <c s="10" r="T427">
         <v>46286</v>
+      </c>
+    </row>
+    <row r="428" ht="17" customHeight="0">
+      <c s="3" r="A428">
+        <v>46303</v>
+      </c>
+      <c s="4" t="inlineStr" r="B428">
+        <is>
+          <t xml:space="preserve">TIB310</t>
+        </is>
+      </c>
+      <c s="3" r="C428">
+        <v>48539</v>
+      </c>
+      <c s="5" r="D428">
+        <v>0.25</v>
+      </c>
+      <c s="4" t="inlineStr" r="E428">
+        <is>
+          <t xml:space="preserve">AU0000171134    </t>
+        </is>
+      </c>
+      <c s="7" r="F428">
+        <v>150000000.0000</v>
+      </c>
+      <c s="7" r="G428">
+        <v>150000000.0000</v>
+      </c>
+      <c s="7" r="H428">
+        <v>590000000.0000</v>
+      </c>
+      <c s="11" r="I428">
+        <v>3.9333</v>
+      </c>
+      <c s="8" r="J428">
+        <v>2.6065</v>
+      </c>
+      <c s="9" r="K428">
+        <v>2.6025</v>
+      </c>
+      <c s="9" r="L428">
+        <v>2.61</v>
+      </c>
+      <c s="9" r="M428">
+        <v>2.63</v>
+      </c>
+      <c s="9" r="N428">
+        <v>2.61575847457627</v>
+      </c>
+      <c s="8" r="O428">
+        <v>2.6115</v>
+      </c>
+      <c s="7" r="P428">
+        <v>43</v>
+      </c>
+      <c s="7" r="Q428">
+        <v>15</v>
+      </c>
+      <c s="7" r="R428">
+        <v>9</v>
+      </c>
+      <c s="7" r="S428">
+        <v>162162450.0000</v>
+      </c>
+      <c s="10" r="T428">
+        <v>46307</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data(aud): daily refresh 2026-10-22T02:46Z
</commit_message>
<xml_diff>
--- a/history/aud/aofm_tib_issuance.xlsx
+++ b/history/aud/aofm_tib_issuance.xlsx
@@ -24901,6 +24901,72 @@
         <v>46307</v>
       </c>
     </row>
+    <row r="429" ht="17" customHeight="0">
+      <c s="3" r="A429">
+        <v>46317</v>
+      </c>
+      <c s="4" t="inlineStr" r="B429">
+        <is>
+          <t xml:space="preserve">TIB311</t>
+        </is>
+      </c>
+      <c s="3" r="C429">
+        <v>49542</v>
+      </c>
+      <c s="5" r="D429">
+        <v>2</v>
+      </c>
+      <c s="4" t="inlineStr" r="E429">
+        <is>
+          <t xml:space="preserve">AU000XCLWAF4    </t>
+        </is>
+      </c>
+      <c s="7" r="F429">
+        <v>150000000.0000</v>
+      </c>
+      <c s="7" r="G429">
+        <v>150000000.0000</v>
+      </c>
+      <c s="7" r="H429">
+        <v>520000000.0000</v>
+      </c>
+      <c s="11" r="I429">
+        <v>3.4666</v>
+      </c>
+      <c s="8" r="J429">
+        <v>2.83733333333333</v>
+      </c>
+      <c s="9" r="K429">
+        <v>2.83</v>
+      </c>
+      <c s="9" r="L429">
+        <v>2.84</v>
+      </c>
+      <c s="9" r="M429">
+        <v>2.8975</v>
+      </c>
+      <c s="9" r="N429">
+        <v>2.84890384615385</v>
+      </c>
+      <c s="8" r="O429">
+        <v>2.8405</v>
+      </c>
+      <c s="7" r="P429">
+        <v>32</v>
+      </c>
+      <c s="7" r="Q429">
+        <v>11</v>
+      </c>
+      <c s="7" r="R429">
+        <v>11</v>
+      </c>
+      <c s="7" r="S429">
+        <v>202084200.0000</v>
+      </c>
+      <c s="10" r="T429">
+        <v>46321</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells>
     <mergeCell ref="A1:G1"/>

</xml_diff>